<commit_message>
Added other questions to questionario_esteso
</commit_message>
<xml_diff>
--- a/assets/questionario_esteso.xlsx
+++ b/assets/questionario_esteso.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6299bfca875a23e8/bandoUniparthenopeSapio/domanmde/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6ABDA4-F01F-4D32-AD1C-CFC8C66A7AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{11217148-A52D-4E31-ACC0-8663F716E21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{450948D2-F6AE-4544-967D-C0A1A48FF49A}"/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="4275" windowWidth="38700" windowHeight="15345" xr2:uid="{9D4E7C91-4F2E-42EB-9306-D9AEE7911042}"/>
+    <workbookView xWindow="2145" yWindow="5010" windowWidth="38700" windowHeight="15345" xr2:uid="{9D4E7C91-4F2E-42EB-9306-D9AEE7911042}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Foglio1!$A$1:$D$65</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="121">
   <si>
     <t>Domanda</t>
   </si>
@@ -277,17 +280,6 @@
     <t>L’impresa utilizza strumenti di analisi organizzativa per monitorare over 50)?</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>Nella ricerca e selezione del personale l’impresa valuta le candidature anche in base all’età tra le seguenti? "esplicita formalmente il requisito",
-        "non inserisce limite ma ne tiene conto",
-        "lo considera per figure con esperienza",
-        "privilegia giovani da formare",
-        "altro",
-        "no"</t>
-  </si>
-  <si>
     <t>Opzioni della risposta multipla ["esplicita formalmente il requisito",
         "non inserisce limite ma ne tiene conto",
         "lo considera per figure con esperienza",
@@ -306,6 +298,221 @@
   </si>
   <si>
     <t>Prodotti/servizi (descrivere mission aziendale [prodotti e servizi e principali linee strategiche/valori aziendali])?</t>
+  </si>
+  <si>
+    <t>19a</t>
+  </si>
+  <si>
+    <t>19b</t>
+  </si>
+  <si>
+    <t>19c</t>
+  </si>
+  <si>
+    <t>19d</t>
+  </si>
+  <si>
+    <t>A quale età un dipendente con qualifica di operaio è considerato professionalmente anziano nell' impresa?</t>
+  </si>
+  <si>
+    <t>A quale età un dipendente con qualifica di impiegato è considerato professionalmente anziano nell' impresa?</t>
+  </si>
+  <si>
+    <t>A quale età un dipendente con qualifica di commerciale è considerato professionalmente anziano nell' impresa?</t>
+  </si>
+  <si>
+    <t>A quale età un dipendente con qualifica di dirigente è considerato professionalmente anziano nell' impresa?</t>
+  </si>
+  <si>
+    <t>Nella ricerca e selezione del personale l’impresa valuta le candidature anche in base all’età?</t>
+  </si>
+  <si>
+    <t>Nella ricerca e selezione del personale l'impresa rivolge una specifica attenzione agli over 50?</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla [
+        "privilegia lavoratori over 50 a rischio espulsione",
+        "prevede percorsi di assunzione dedicati",
+        "attiva contatti con agenzie specializzate",
+        "privilegia over 50 con incentivi/sussidi",
+        "altro",
+        "no"
+      ]. Non prevedere altre parole o caratteri</t>
+  </si>
+  <si>
+    <t>La sua impresa attua iniziative specifiche di age management?</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, Descrivere l’esperienza progettuale di age management</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, descrivere Da quale esigenza/criticità è nata l’iniziativa?</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, descrivere Da chi e con quale modalità è stata progettata l’iniziativa?</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, descrivere Elementi di forza/aspetti positivi dell’iniziativa</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, descrivere Elementi di debolezza/criticità ed eventuali soluzioni adottate</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, descrivere Risultati ottenuti dall’iniziativa</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, descrivere  se L’iniziativa è sostenibile in termini di risorse e costi/benefici?</t>
+  </si>
+  <si>
+    <t>In merito alle esperienze specifiche di age management, se ci sono, descrivere se l'iniziativa è stata o sarà replicata nella stessa impresa, in altre sedi aziendali o in altre imprese dello stesso gruppo, o se non sarà replicata</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla [
+        "nella stessa impresa",
+        "in altre sedi aziendali",
+        "in altre imprese del gruppo",
+        "no"
+      ]</t>
+  </si>
+  <si>
+    <t>Azioni specifiche per sviluppare competenze dei lavoratori over 50</t>
+  </si>
+  <si>
+    <t>Qual è il Codice Fiscale / numero di Partita Iva ( P.IVA) dell' azienda?</t>
+  </si>
+  <si>
+    <t>Rispondi solo con il codice alfanumerico. non inserire ragionamento o costruzioni di una frase. Rispondi in maniera diretta e specifica</t>
+  </si>
+  <si>
+    <t>In merito ai Percorsi di Carriera, Sono previste strategie per sostenere motivazione e produttività lungo tutto l’arco lavorativo?</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla: [
+        "formazione interna",
+        "formazione esterna",
+        "corsi per lavoratori in mobilità",
+        "mentoring/tutoring/coaching",
+        "scambi formativi",
+        "percorsi di certificazione competenze",
+        "supporto a progetti personali",
+        "altro",
+        "no"
+      ]</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla: ["incentivi",
+        "premi",
+        "riconoscimenti",
+        "coinvolgimento dei lavoratori",
+        "indagini periodiche",
+        "proposte formative",
+        "dialogo intergenerazionale",
+        "people caring",
+        "riprogettazione dei compiti",
+        "altro",
+        "no"]</t>
+  </si>
+  <si>
+    <t>In merito ai Percorsi di Carriera, Sono previste Azioni per lo sviluppo dei percorsi di carriera?</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipola: [
+        "valorizzazione competenze/esperienza",
+        "cambio ruolo/mansioni",
+        "ruolo di maestro/tutor",
+        "strumenti per identificare abilità e potenziale",
+        "ri-orientamento professionale",
+        "altro",
+        "no"
+      ]</t>
+  </si>
+  <si>
+    <t>In merito ai Percorsi di Carriera, Quale aspetto è primario nell’assegnazione di mansioni strategiche?</t>
+  </si>
+  <si>
+    <t>In merito ai Percorsi di Carriera, L’impresa favorisce la permanenza degli over 50 con modalità organizzative innovative?</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla: [ "esperienza",
+        "competenze",
+        "titolo di studio",
+        "anzianità aziendale",
+        "altro"
+      ]</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla: [
+        "flessibilità orari/tempi",
+        "telelavoro",
+        "formazione ai giovani in sostituzione pensionamento anticipato",
+        "team working / job rotation",
+        "nuove tecnologie + formazione",
+        "pratiche di conciliazione",
+        "iniziative di fidelizzazione",
+        "altro",
+        "no"
+      ]</t>
+  </si>
+  <si>
+    <t>In merito ai Percorsi di Carriera, Attraverso la contrattazione di secondo livello sono attivate misure per i lavoratori over 50?</t>
+  </si>
+  <si>
+    <t>In materia di Tutela della salute dei lavoratori, sono previsti Interventi specifici per la tutela della salute psico-fisica dei lavoratori over 50?</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla: [
+        "controlli medici periodici differenziati",
+        "consulenza su salute e sicurezza",
+        "campagne sensibilizzazione sicurezza sul lavoro",
+        "campagne sensibilizzazione salute generale",
+        "strumenti monitoraggio salute (es. WAI)",
+        "affiancamento giovani-anziani",
+        "sostituzione attrezzature obsolete",
+        "spazi ricreativi",
+        "miglioramento ambiente lavorativo",
+        "ergonomia postazioni",
+        "attività/servizi benessere psico-fisico",
+        "periodi di congedo aggiuntivi",
+        "accompagnamento al reinserimento lavorativo",
+        "valutazione rischi",
+        "altro",
+        "no"</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla:  [
+        "assistenza pre-pensionistica",
+        "riduzioni orario",
+        "uscita collegata a entrata giovani",
+        "creazione società di consulenza",
+        "supporto attività associative/volontariato",
+        "altro",
+        "no"
+      ]</t>
+  </si>
+  <si>
+    <t>Sono previsti Strumenti di sostegno all’uscita graduale e al pensionamento?</t>
+  </si>
+  <si>
+    <t>Sono avvenuti casi di pensionamento e riassunzione di ex dipendenti?</t>
+  </si>
+  <si>
+    <t>Negli ultimi tre anni l’impresa ha effettuato cessazioni o utilizzato ammortizzatori sociali?</t>
+  </si>
+  <si>
+    <t>Opzioni della risposta multipla: [
+        "fine contratto a termine",
+        "pre-pensionamenti",
+        "richiesta dimissioni",
+        "iniziative di outplacement",
+        "licenziamenti",
+        "contratti di solidarietà",
+        "CIG ordinaria",
+        "CIG straordinaria",
+        "mobilità"
+      ]</t>
+  </si>
+  <si>
+    <t>Rispondi in maniera aperta ma concisa.</t>
   </si>
 </sst>
 </file>
@@ -362,6 +569,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -681,11 +892,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A50ED679-D331-4C4E-A2B2-164B5F3F2531}">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.28515625" customWidth="1"/>
-    <col min="3" max="3" width="244" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="162.42578125" customWidth="1"/>
     <col min="4" max="4" width="115.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -705,27 +916,27 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -733,13 +944,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -747,13 +958,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -761,52 +972,55 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>78</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
         <v>3</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
         <v>18</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
       </c>
       <c r="D9" t="s">
         <v>29</v>
@@ -814,41 +1028,41 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
         <v>20</v>
       </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="D11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" t="s">
         <v>21</v>
-      </c>
-      <c r="D11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" t="s">
-        <v>22</v>
       </c>
       <c r="D12" t="s">
         <v>29</v>
@@ -856,41 +1070,41 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
         <v>23</v>
       </c>
-      <c r="D13" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="D14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B14" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="B15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
         <v>24</v>
-      </c>
-      <c r="D14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" t="s">
-        <v>25</v>
       </c>
       <c r="D15" t="s">
         <v>29</v>
@@ -898,10 +1112,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D16" t="s">
         <v>29</v>
@@ -909,83 +1126,83 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>17</v>
       </c>
-      <c r="B17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="B18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
         <v>26</v>
       </c>
-      <c r="D17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18">
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>14</v>
       </c>
-      <c r="B18" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" t="s">
         <v>32</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A19">
+    <row r="20" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>15</v>
       </c>
-      <c r="B19" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A20">
+    <row r="21" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>16</v>
       </c>
-      <c r="B20" t="s">
-        <v>5</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="B21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B22" t="s">
         <v>5</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D22" t="s">
         <v>29</v>
@@ -993,13 +1210,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" t="s">
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
@@ -1007,13 +1224,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B24" t="s">
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
         <v>29</v>
@@ -1021,13 +1238,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B25" t="s">
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
         <v>29</v>
@@ -1035,13 +1252,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B26" t="s">
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D26" t="s">
         <v>29</v>
@@ -1049,13 +1266,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B27" t="s">
         <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
@@ -1063,13 +1280,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B28" t="s">
         <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D28" t="s">
         <v>29</v>
@@ -1077,13 +1294,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D29" t="s">
         <v>29</v>
@@ -1091,13 +1308,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="D30" t="s">
         <v>29</v>
@@ -1105,13 +1322,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="D31" t="s">
         <v>29</v>
@@ -1119,13 +1336,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D32" t="s">
         <v>29</v>
@@ -1133,13 +1350,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" t="s">
         <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D33" t="s">
         <v>29</v>
@@ -1147,28 +1364,27 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B34" t="s">
         <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D34" t="s">
         <v>29</v>
       </c>
-      <c r="E34" s="2"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B35" t="s">
         <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D35" t="s">
         <v>29</v>
@@ -1177,13 +1393,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B36" t="s">
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D36" t="s">
         <v>29</v>
@@ -1192,13 +1408,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B37" t="s">
         <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D37" t="s">
         <v>29</v>
@@ -1207,127 +1423,399 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>60</v>
+      </c>
+      <c r="D38" t="s">
+        <v>29</v>
+      </c>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>72</v>
       </c>
-      <c r="B38" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="B39" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39" t="s">
         <v>61</v>
       </c>
-      <c r="D38" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>18</v>
-      </c>
-      <c r="B39" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" t="s">
-        <v>73</v>
-      </c>
       <c r="D39" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" t="s">
+        <v>73</v>
+      </c>
+      <c r="D40" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>79</v>
+      </c>
+      <c r="B41" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" t="s">
+        <v>83</v>
+      </c>
+      <c r="D41" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>80</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>84</v>
+      </c>
+      <c r="D42" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>81</v>
+      </c>
+      <c r="B43" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43" t="s">
+        <v>85</v>
+      </c>
+      <c r="D43" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" t="s">
+        <v>5</v>
+      </c>
+      <c r="C44" t="s">
+        <v>86</v>
+      </c>
+      <c r="D44" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>20</v>
+      </c>
+      <c r="B45" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>20</v>
-      </c>
-      <c r="B41" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42">
+    <row r="46" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+      <c r="A46">
         <v>21</v>
       </c>
-      <c r="B42" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>22</v>
-      </c>
-      <c r="B43" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>23</v>
-      </c>
-      <c r="B44" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>24</v>
-      </c>
-      <c r="B45" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>25</v>
-      </c>
       <c r="B46" t="s">
         <v>5</v>
+      </c>
+      <c r="C46" t="s">
+        <v>88</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B47" t="s">
         <v>5</v>
+      </c>
+      <c r="C47" t="s">
+        <v>90</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
+        <v>23</v>
+      </c>
+      <c r="B48" t="s">
+        <v>5</v>
+      </c>
+      <c r="C48" t="s">
+        <v>91</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>24</v>
+      </c>
+      <c r="B49" t="s">
+        <v>5</v>
+      </c>
+      <c r="C49" t="s">
+        <v>92</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>25</v>
+      </c>
+      <c r="B50" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50" t="s">
+        <v>93</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>26</v>
+      </c>
+      <c r="B51" t="s">
+        <v>5</v>
+      </c>
+      <c r="C51" t="s">
+        <v>94</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
         <v>27</v>
       </c>
-      <c r="B48" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49">
+      <c r="B52" t="s">
+        <v>5</v>
+      </c>
+      <c r="C52" t="s">
+        <v>95</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
         <v>28</v>
       </c>
-      <c r="B49" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>29</v>
-      </c>
-      <c r="B50" t="s">
-        <v>5</v>
+      <c r="B53" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53" t="s">
+        <v>96</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>29</v>
+      </c>
+      <c r="B54" t="s">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s">
+        <v>97</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>30</v>
+      </c>
+      <c r="B55" t="s">
+        <v>5</v>
+      </c>
+      <c r="C55" t="s">
+        <v>98</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>31</v>
+      </c>
+      <c r="B56" t="s">
+        <v>5</v>
+      </c>
+      <c r="C56" t="s">
+        <v>100</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>32</v>
+      </c>
+      <c r="B57" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57" t="s">
+        <v>103</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="135" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>33</v>
+      </c>
+      <c r="B58" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" t="s">
+        <v>106</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>34</v>
+      </c>
+      <c r="B59" t="s">
+        <v>5</v>
+      </c>
+      <c r="C59" t="s">
+        <v>108</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>35</v>
+      </c>
+      <c r="B60" t="s">
+        <v>5</v>
+      </c>
+      <c r="C60" t="s">
+        <v>109</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>36</v>
+      </c>
+      <c r="B61" t="s">
+        <v>5</v>
+      </c>
+      <c r="C61" t="s">
+        <v>112</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="255" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>37</v>
+      </c>
+      <c r="B62" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" t="s">
+        <v>113</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="135" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>38</v>
+      </c>
+      <c r="B63" t="s">
+        <v>5</v>
+      </c>
+      <c r="C63" t="s">
+        <v>116</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>39</v>
+      </c>
+      <c r="B64" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64" t="s">
+        <v>117</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>40</v>
+      </c>
+      <c r="B65" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" t="s">
+        <v>118</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D65" xr:uid="{A50ED679-D331-4C4E-A2B2-164B5F3F2531}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>